<commit_message>
chore: daily reconciliation 2026-05-06
</commit_message>
<xml_diff>
--- a/output/recon_2026-05-06.xlsx
+++ b/output/recon_2026-05-06.xlsx
@@ -573,13 +573,13 @@
         <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>57.1941763</v>
+        <v>57.19418722</v>
       </c>
       <c r="E3" t="n">
-        <v>56.1941763</v>
+        <v>56.19418722</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>57.1941763</v>
+        <v>57.19418722</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>67500</v>
@@ -639,19 +639,19 @@
         <v>60</v>
       </c>
       <c r="D5" t="n">
-        <v>120133.627066</v>
+        <v>120133.877066</v>
       </c>
       <c r="E5" t="n">
-        <v>-866.372934</v>
+        <v>-866.122934</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.992839893107438</v>
+        <v>0.9928419592231404</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>866.372934</v>
+        <v>866.122934</v>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>57.1941763</v>
+        <v>57.19418722</v>
       </c>
     </row>
     <row r="3">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>120133.627066</v>
+        <v>120133.877066</v>
       </c>
     </row>
     <row r="6">

</xml_diff>